<commit_message>
Week 3 Update last
</commit_message>
<xml_diff>
--- a/cohort 2026/template_MADIEGA_files/Energy_Supply_System_2026.xlsx
+++ b/cohort 2026/template_MADIEGA_files/Energy_Supply_System_2026.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\L3_BIT\Bachelor\infineon\MADIEGA_S\template_MADIEGA_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00519C3-4A8D-417B-8CB2-60E7C3F48ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DBEF72-0CA7-4DD7-BB9F-6884734A8C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Solar PV power plant" sheetId="6" r:id="rId1"/>
     <sheet name="Solar &amp; Energy Systems" sheetId="7" r:id="rId2"/>
-    <sheet name="Energy Supply Systems — Aida" sheetId="9" r:id="rId3"/>
-    <sheet name="ENERGY SUPPLY SUMMARY" sheetId="11" r:id="rId4"/>
+    <sheet name="Energy Systems" sheetId="9" r:id="rId3"/>
+    <sheet name="ENERGY SYSTEM SUMMARY" sheetId="11" r:id="rId4"/>
+    <sheet name="TEAM SUMMARY — Energy System" sheetId="12" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -180,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="511">
   <si>
     <t>Years</t>
   </si>
@@ -1492,6 +1493,370 @@
   <si>
     <t>Panel failure, low battery, generator activation, grid outage</t>
   </si>
+  <si>
+    <t>Abdoul (base)</t>
+  </si>
+  <si>
+    <t>3 kW × 5h</t>
+  </si>
+  <si>
+    <t>Aida (new)</t>
+  </si>
+  <si>
+    <t>Water Supply 2026 ,  validated by real data (20 m³/day ÷ 4 m³/h)</t>
+  </si>
+  <si>
+    <t>Energy Consumption (Revised)</t>
+  </si>
+  <si>
+    <t>Misc.</t>
+  </si>
+  <si>
+    <t>Extended (Aida)</t>
+  </si>
+  <si>
+    <t>7.5</t>
+  </si>
+  <si>
+    <t>11.5</t>
+  </si>
+  <si>
+    <t>34.0</t>
+  </si>
+  <si>
+    <t>184.0</t>
+  </si>
+  <si>
+    <t>634.0</t>
+  </si>
+  <si>
+    <t>3,034.0</t>
+  </si>
+  <si>
+    <t>PV Sizing (Revised)</t>
+  </si>
+  <si>
+    <t>6.87</t>
+  </si>
+  <si>
+    <t>58.4</t>
+  </si>
+  <si>
+    <t>0.0058</t>
+  </si>
+  <si>
+    <t>37.17</t>
+  </si>
+  <si>
+    <t>316.0</t>
+  </si>
+  <si>
+    <t>0.0316</t>
+  </si>
+  <si>
+    <t>128.08</t>
+  </si>
+  <si>
+    <t>1,088.7</t>
+  </si>
+  <si>
+    <t>0.1089</t>
+  </si>
+  <si>
+    <t>613.13</t>
+  </si>
+  <si>
+    <t>5,211.6</t>
+  </si>
+  <si>
+    <t>0.5212</t>
+  </si>
+  <si>
+    <t>Battery Sizing (Revised)</t>
+  </si>
+  <si>
+    <t>11.33</t>
+  </si>
+  <si>
+    <t>12.59</t>
+  </si>
+  <si>
+    <t>15.74</t>
+  </si>
+  <si>
+    <t>61.33</t>
+  </si>
+  <si>
+    <t>68.15</t>
+  </si>
+  <si>
+    <t>85.19</t>
+  </si>
+  <si>
+    <t>211.33</t>
+  </si>
+  <si>
+    <t>234.81</t>
+  </si>
+  <si>
+    <t>293.52</t>
+  </si>
+  <si>
+    <t>1,011.33</t>
+  </si>
+  <si>
+    <t>1,123.70</t>
+  </si>
+  <si>
+    <t>1,404.63</t>
+  </si>
+  <si>
+    <t>CAPEX (Revised)</t>
+  </si>
+  <si>
+    <t>1,297,608</t>
+  </si>
+  <si>
+    <t>Tracking Comparison (Revised)</t>
+  </si>
+  <si>
+    <t>6.98 kWp</t>
+  </si>
+  <si>
+    <t>5.51 kWp</t>
+  </si>
+  <si>
+    <t>20% fewer panels</t>
+  </si>
+  <si>
+    <t>~40,275</t>
+  </si>
+  <si>
+    <t>~39,380</t>
+  </si>
+  <si>
+    <t>Tracking remains cheaper</t>
+  </si>
+  <si>
+    <t>12,410 kWh/yr</t>
+  </si>
+  <si>
+    <t>Base 34 kWh/day × 365</t>
+  </si>
+  <si>
+    <t>Annual Savings (at 0.40 $/kWh)</t>
+  </si>
+  <si>
+    <t>4,964 $/yr</t>
+  </si>
+  <si>
+    <t>Payback</t>
+  </si>
+  <si>
+    <t>~8.1 years</t>
+  </si>
+  <si>
+    <t>~7.9 years</t>
+  </si>
+  <si>
+    <t>Consistent with overall ROI calculation</t>
+  </si>
+  <si>
+    <t>9.5 kWh/day</t>
+  </si>
+  <si>
+    <t>Annual Usage</t>
+  </si>
+  <si>
+    <t>Annual Cost</t>
+  </si>
+  <si>
+    <t>Annual Emissions</t>
+  </si>
+  <si>
+    <t>1,080 kg CO₂/year</t>
+  </si>
+  <si>
+    <t>+ Generator</t>
+  </si>
+  <si>
+    <t>Total Emissions</t>
+  </si>
+  <si>
+    <t>620.5</t>
+  </si>
+  <si>
+    <t>1,700.5</t>
+  </si>
+  <si>
+    <t>86.8%</t>
+  </si>
+  <si>
+    <t>11,570.5</t>
+  </si>
+  <si>
+    <t>12,650.5</t>
+  </si>
+  <si>
+    <t>89.1%</t>
+  </si>
+  <si>
+    <t>1,107,410</t>
+  </si>
+  <si>
+    <t>55,370.5</t>
+  </si>
+  <si>
+    <t>56,450.5</t>
+  </si>
+  <si>
+    <t>89.</t>
+  </si>
+  <si>
+    <t>Dried Output (kg/day)</t>
+  </si>
+  <si>
+    <t>CO₂/kg dried mango</t>
+  </si>
+  <si>
+    <t>16.5</t>
+  </si>
+  <si>
+    <t>0.737</t>
+  </si>
+  <si>
+    <t>0.525</t>
+  </si>
+  <si>
+    <t>0.469</t>
+  </si>
+  <si>
+    <r>
+      <t>5 h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(corrected, was 4h)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pump </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(corrected)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Generator Backup Sizing </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(added)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Carbon Footprint Calculator </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(added)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>72.6%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(vs 71.8% before)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CO₂ per kg dried mango</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(for connection SANON — Product Transformation)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1501,7 +1866,7 @@
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="48" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1788,6 +2153,21 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1962,7 +2342,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2269,6 +2649,78 @@
     <xf numFmtId="10" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="28" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2278,9 +2730,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2296,72 +2745,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="28" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2384,85 +2767,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="133">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
+  <dxfs count="191">
     <dxf>
       <font>
         <b val="0"/>
@@ -2477,8 +2795,29 @@
         <sz val="14"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2494,8 +2833,10 @@
         <sz val="14"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2511,8 +2852,10 @@
         <sz val="14"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2526,10 +2869,31 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="14"/>
-        <color rgb="FF000000"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2545,74 +2909,10 @@
         <sz val="14"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2625,13 +2925,32 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2644,13 +2963,13 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2663,13 +2982,222 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2682,13 +3210,13 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2701,6 +3229,418 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
@@ -4601,6 +5541,541 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
         <family val="1"/>
@@ -4640,294 +6115,415 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9DC580F5-1ABC-41E0-8B0A-CB73A01DD91E}" name="Table4" displayName="Table4" ref="H10:J15" totalsRowShown="0" headerRowDxfId="132" dataDxfId="131">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9DC580F5-1ABC-41E0-8B0A-CB73A01DD91E}" name="Table4" displayName="Table4" ref="H10:J15" totalsRowShown="0" headerRowDxfId="161" dataDxfId="160">
   <autoFilter ref="H10:J15" xr:uid="{9DC580F5-1ABC-41E0-8B0A-CB73A01DD91E}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B8E2BFC1-4365-44A7-B0ED-19B68A88E45F}" name="Parameter" dataDxfId="130"/>
-    <tableColumn id="2" xr3:uid="{B0480422-1F14-44CC-B337-6BF7542943CB}" name="Value" dataDxfId="129"/>
-    <tableColumn id="3" xr3:uid="{B8F2FB03-C6E8-4B7C-BA40-B1442FF77348}" name="Source" dataDxfId="128"/>
+    <tableColumn id="1" xr3:uid="{B8E2BFC1-4365-44A7-B0ED-19B68A88E45F}" name="Parameter" dataDxfId="159"/>
+    <tableColumn id="2" xr3:uid="{B0480422-1F14-44CC-B337-6BF7542943CB}" name="Value" dataDxfId="158"/>
+    <tableColumn id="3" xr3:uid="{B8F2FB03-C6E8-4B7C-BA40-B1442FF77348}" name="Source" dataDxfId="157"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{EDE741E4-62D0-47ED-8551-F326AAEF0FB1}" name="Table13" displayName="Table13" ref="L8:N12" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{EDE741E4-62D0-47ED-8551-F326AAEF0FB1}" name="Table13" displayName="Table13" ref="L8:N12" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
   <autoFilter ref="L8:N12" xr:uid="{EDE741E4-62D0-47ED-8551-F326AAEF0FB1}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6E3284C9-6692-4728-9AF9-7E8BF4D6F4BA}" name="Parameter" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{2FA1ACCE-702A-4041-BEF5-98EE436367CA}" name="Value" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{5AD9B4EB-8369-4D93-AE2E-8BE158293515}" name="Source" dataDxfId="75"/>
+    <tableColumn id="1" xr3:uid="{6E3284C9-6692-4728-9AF9-7E8BF4D6F4BA}" name="Parameter" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{2FA1ACCE-702A-4041-BEF5-98EE436367CA}" name="Value" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{5AD9B4EB-8369-4D93-AE2E-8BE158293515}" name="Source" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7FCF354-D5F8-41BF-82BB-CE15410B69BF}" name="Table14" displayName="Table14" ref="R8:T13" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7FCF354-D5F8-41BF-82BB-CE15410B69BF}" name="Table14" displayName="Table14" ref="R8:T13" totalsRowShown="0" headerRowDxfId="103" dataDxfId="102">
   <autoFilter ref="R8:T13" xr:uid="{B7FCF354-D5F8-41BF-82BB-CE15410B69BF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6B4F370E-8917-4DD6-A0A9-8DAB27AD166F}" name="Parameter" dataDxfId="72"/>
-    <tableColumn id="2" xr3:uid="{41245AEB-AE5B-4C79-AC34-E756B56FB9F5}" name="Value" dataDxfId="71"/>
-    <tableColumn id="3" xr3:uid="{86765024-F6E8-4CA8-B17A-DD71F18EB5E0}" name="Source" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{6B4F370E-8917-4DD6-A0A9-8DAB27AD166F}" name="Parameter" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{41245AEB-AE5B-4C79-AC34-E756B56FB9F5}" name="Value" dataDxfId="100"/>
+    <tableColumn id="3" xr3:uid="{86765024-F6E8-4CA8-B17A-DD71F18EB5E0}" name="Source" dataDxfId="99"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F9491EAD-8F3A-4365-A4D1-1004A562ECDD}" name="Table516" displayName="Table516" ref="X8:AA12" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F9491EAD-8F3A-4365-A4D1-1004A562ECDD}" name="Table516" displayName="Table516" ref="X8:AA12" totalsRowShown="0" headerRowDxfId="98" dataDxfId="97">
   <autoFilter ref="X8:AA12" xr:uid="{F9491EAD-8F3A-4365-A4D1-1004A562ECDD}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3A42ACD2-4734-4B9A-94A0-C80983D67309}" name="Scenario" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{8F8D7EE1-39A0-4FC4-8461-3F528B815119}" name="Original Total (Abdoul)" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{66BB0B2A-040B-45C2-9C28-4214DC283B19}" name="+ Extended Load" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{56589B10-F911-4E8A-B1CA-504335936EC8}" name="New TOTAL" dataDxfId="64"/>
+    <tableColumn id="1" xr3:uid="{3A42ACD2-4734-4B9A-94A0-C80983D67309}" name="Scenario" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{8F8D7EE1-39A0-4FC4-8461-3F528B815119}" name="Original Total (Abdoul)" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{66BB0B2A-040B-45C2-9C28-4214DC283B19}" name="+ Extended Load" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{56589B10-F911-4E8A-B1CA-504335936EC8}" name="New TOTAL" dataDxfId="93"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD31F287-FA05-4C48-822B-D9810C165457}" name="Table62" displayName="Table62" ref="E36:J40" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FD31F287-FA05-4C48-822B-D9810C165457}" name="Table62" displayName="Table62" ref="E36:J40" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
   <autoFilter ref="E36:J40" xr:uid="{FD31F287-FA05-4C48-822B-D9810C165457}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6BBC6055-379C-4BBA-BB3F-9D56898B2B69}" name="Scenario" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{FEF3E7B0-C50E-4078-8876-D007376BE2D2}" name="Energy (kWh/day)" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{00C6F3C3-9275-4EF1-A0D5-2D458360C194}" name="PV required (kWp)" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{DF78E3C6-03E9-4978-9D33-EC5D975D0152}" name="No. of 400W panels" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{E1A0656B-BA9B-43FA-BA75-61BC4B4FDCBA}" name="Area (m²)" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{3DF14469-183B-4F24-B281-5700B21CE8C5}" name="Area (ha)" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{6BBC6055-379C-4BBA-BB3F-9D56898B2B69}" name="Scenario" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{FEF3E7B0-C50E-4078-8876-D007376BE2D2}" name="Energy (kWh/day)" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{00C6F3C3-9275-4EF1-A0D5-2D458360C194}" name="PV required (kWp)" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{DF78E3C6-03E9-4978-9D33-EC5D975D0152}" name="No. of 400W panels" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{E1A0656B-BA9B-43FA-BA75-61BC4B4FDCBA}" name="Area (m²)" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{3DF14469-183B-4F24-B281-5700B21CE8C5}" name="Area (ha)" dataDxfId="85"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{360DA6B4-1904-4E4B-A18F-B6BC9A0CC6C2}" name="Table73" displayName="Table73" ref="F47:I51" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{360DA6B4-1904-4E4B-A18F-B6BC9A0CC6C2}" name="Table73" displayName="Table73" ref="F47:I51" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
   <autoFilter ref="F47:I51" xr:uid="{360DA6B4-1904-4E4B-A18F-B6BC9A0CC6C2}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{93E65EBA-3C9A-48BF-9B9C-6E0E5A6C9F80}" name="Scenario" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{3005B769-2A1A-43B9-A1B0-36C96C0369A3}" name="Energy/8h (kWh)" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{879BCFE5-4855-4794-8E4C-54D2EDDBF609}" name="With losses (kWh)" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{03853E53-FEB8-4B01-B0E0-F6F37F191246}" name="Nominal capacity (kWh)" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{93E65EBA-3C9A-48BF-9B9C-6E0E5A6C9F80}" name="Scenario" dataDxfId="82"/>
+    <tableColumn id="2" xr3:uid="{3005B769-2A1A-43B9-A1B0-36C96C0369A3}" name="Energy/8h (kWh)" dataDxfId="81"/>
+    <tableColumn id="3" xr3:uid="{879BCFE5-4855-4794-8E4C-54D2EDDBF609}" name="With losses (kWh)" dataDxfId="80"/>
+    <tableColumn id="4" xr3:uid="{03853E53-FEB8-4B01-B0E0-F6F37F191246}" name="Nominal capacity (kWh)" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A8B3987-75F4-4183-9401-BF164DD53776}" name="Table84" displayName="Table84" ref="F58:I62" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A8B3987-75F4-4183-9401-BF164DD53776}" name="Table84" displayName="Table84" ref="F58:I62" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="F58:I62" xr:uid="{6A8B3987-75F4-4183-9401-BF164DD53776}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{8A7F1C9B-2D31-41DE-B0F5-4D77E06EDC53}" name="Scenario" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{D3103AFF-309C-4D14-AA6A-9DC1E0AAA856}" name="PV cost ($)" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{1F2780AA-1518-451E-ACE9-07D4AB068DA9}" name="Battery ($)" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{10ABABA8-316E-4FCB-8E78-903E7B910CF5}" name="Subtotal (excl. inverter)" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{8A7F1C9B-2D31-41DE-B0F5-4D77E06EDC53}" name="Scenario" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{D3103AFF-309C-4D14-AA6A-9DC1E0AAA856}" name="PV cost ($)" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{1F2780AA-1518-451E-ACE9-07D4AB068DA9}" name="Battery ($)" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{10ABABA8-316E-4FCB-8E78-903E7B910CF5}" name="Subtotal (excl. inverter)" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8F1CAA6F-D84A-4725-9C33-E68157DCC17C}" name="Table16" displayName="Table16" ref="B69:E73" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{8F1CAA6F-D84A-4725-9C33-E68157DCC17C}" name="Table16" displayName="Table16" ref="B69:E73" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
   <autoFilter ref="B69:E73" xr:uid="{8F1CAA6F-D84A-4725-9C33-E68157DCC17C}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D1B0ADE3-9E63-4869-AF65-8B5CE13F763A}" name="Parameter" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{1CD0E490-FEF6-42EC-8E97-8B1C4E841698}" name="Fixed-Tilt" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{EB3CD6E1-4606-456B-B452-3474CAA5B5FF}" name="Tracking" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{F0AC3825-0CE1-4987-883F-C363BA0B6528}" name="Comment" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{D1B0ADE3-9E63-4869-AF65-8B5CE13F763A}" name="Parameter" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{1CD0E490-FEF6-42EC-8E97-8B1C4E841698}" name="Fixed-Tilt" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{EB3CD6E1-4606-456B-B452-3474CAA5B5FF}" name="Tracking" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{F0AC3825-0CE1-4987-883F-C363BA0B6528}" name="Comment" dataDxfId="67"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CE18C287-09E0-4184-B089-3C4DD91C2D12}" name="Table17" displayName="Table17" ref="B78:D87" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{CE18C287-09E0-4184-B089-3C4DD91C2D12}" name="Table17" displayName="Table17" ref="B78:D87" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
   <autoFilter ref="B78:D87" xr:uid="{CE18C287-09E0-4184-B089-3C4DD91C2D12}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B082F0D0-CC72-4606-ACAB-426F9469051A}" name="Parameter" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{358A5A4C-ACE2-473A-A823-EA225FD507BB}" name="Value" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{1DC3F3EF-EC1E-4AAA-AE27-227457BAFF5C}" name="Comment" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{B082F0D0-CC72-4606-ACAB-426F9469051A}" name="Parameter" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{358A5A4C-ACE2-473A-A823-EA225FD507BB}" name="Value" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{1DC3F3EF-EC1E-4AAA-AE27-227457BAFF5C}" name="Comment" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{B5F53602-6FB0-400A-89F8-4715114100C6}" name="Table1019" displayName="Table1019" ref="B92:D95" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{B5F53602-6FB0-400A-89F8-4715114100C6}" name="Table1019" displayName="Table1019" ref="B92:D95" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="B92:D95" xr:uid="{B5F53602-6FB0-400A-89F8-4715114100C6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{155709BB-DC21-4C44-92A3-AE254DE9161B}" name="Parameter" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{EDEA325A-F1BA-442E-9A16-9811338C546D}" name="Value" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{F8584D6F-CDD7-47CF-8DD6-625B8AD3C323}" name="Comment" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{155709BB-DC21-4C44-92A3-AE254DE9161B}" name="Parameter" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{EDEA325A-F1BA-442E-9A16-9811338C546D}" name="Value" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{F8584D6F-CDD7-47CF-8DD6-625B8AD3C323}" name="Comment" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{6B511EB4-3A20-4056-AD40-F77DE9142A5D}" name="Table1123" displayName="Table1123" ref="F92:L96" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{6B511EB4-3A20-4056-AD40-F77DE9142A5D}" name="Table1123" displayName="Table1123" ref="F92:L96" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="F92:L96" xr:uid="{6B511EB4-3A20-4056-AD40-F77DE9142A5D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B85A3D86-7257-4ABF-A3CA-29CB58A9671B}" name="Scenario" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{21BE9CAE-B2F9-4FC7-84FF-F6194455FBF3}" name="Annual Production (kWh/yr)" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{543D5FE1-4BE3-4EC8-BEA6-969B01549EC2}" name="PV Emissions (kg CO₂/yr)" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{553ED81B-4207-4DA8-A747-09B1C30F7E62}" name="Grid Equivalent (kg CO₂/yr)" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{79398174-75C3-4B1D-8C7A-2ADF3EDB1D51}" name="+ Generator (kg CO₂/yr)" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{F6020B91-A020-4324-A7AE-D648CD863DB9}" name="Total System Emissions" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{ACFB10EC-4DA6-4F85-BCDA-714D1961EA83}" name="Reduction vs Grid" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{B85A3D86-7257-4ABF-A3CA-29CB58A9671B}" name="Scenario" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{21BE9CAE-B2F9-4FC7-84FF-F6194455FBF3}" name="Annual Production (kWh/yr)" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{543D5FE1-4BE3-4EC8-BEA6-969B01549EC2}" name="PV Emissions (kg CO₂/yr)" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{553ED81B-4207-4DA8-A747-09B1C30F7E62}" name="Grid Equivalent (kg CO₂/yr)" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{79398174-75C3-4B1D-8C7A-2ADF3EDB1D51}" name="+ Generator (kg CO₂/yr)" dataDxfId="50"/>
+    <tableColumn id="6" xr3:uid="{F6020B91-A020-4324-A7AE-D648CD863DB9}" name="Total System Emissions" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{ACFB10EC-4DA6-4F85-BCDA-714D1961EA83}" name="Reduction vs Grid" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E2C190AF-C450-412C-A708-8EF4A2550042}" name="Table5" displayName="Table5" ref="P3:S7" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E2C190AF-C450-412C-A708-8EF4A2550042}" name="Table5" displayName="Table5" ref="P3:S7" totalsRowShown="0" headerRowDxfId="156" dataDxfId="155">
   <autoFilter ref="P3:S7" xr:uid="{E2C190AF-C450-412C-A708-8EF4A2550042}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2C1FFB2F-AF3F-4A27-8F50-7C75FFC47273}" name="Scenario" dataDxfId="125"/>
-    <tableColumn id="2" xr3:uid="{0A9753BB-E417-4E7A-B6B1-B43D2AC56C0D}" name="Original Total (Abdoul)" dataDxfId="124"/>
-    <tableColumn id="3" xr3:uid="{7A31C4ED-8DC7-4547-A50A-2BB3BB98FE95}" name="+ Extended Load" dataDxfId="123"/>
-    <tableColumn id="4" xr3:uid="{D80A5B79-3343-4BAC-A3FD-035C50525C20}" name="New TOTAL" dataDxfId="122"/>
+    <tableColumn id="1" xr3:uid="{2C1FFB2F-AF3F-4A27-8F50-7C75FFC47273}" name="Scenario" dataDxfId="154"/>
+    <tableColumn id="2" xr3:uid="{0A9753BB-E417-4E7A-B6B1-B43D2AC56C0D}" name="Original Total (Abdoul)" dataDxfId="153"/>
+    <tableColumn id="3" xr3:uid="{7A31C4ED-8DC7-4547-A50A-2BB3BB98FE95}" name="+ Extended Load" dataDxfId="152"/>
+    <tableColumn id="4" xr3:uid="{D80A5B79-3343-4BAC-A3FD-035C50525C20}" name="New TOTAL" dataDxfId="151"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{97FE031A-1963-4B47-BEF7-83E334D3D081}" name="Table924" displayName="Table924" ref="B101:C106" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{97FE031A-1963-4B47-BEF7-83E334D3D081}" name="Table924" displayName="Table924" ref="B101:C106" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="B101:C106" xr:uid="{97FE031A-1963-4B47-BEF7-83E334D3D081}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1DC614B9-B28F-4C7E-AB73-A6A06D252743}" name="Screen" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{F5155985-C3D6-43DC-A9BA-7ABF77D8A2BB}" name="Content" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{1DC614B9-B28F-4C7E-AB73-A6A06D252743}" name="Screen" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{F5155985-C3D6-43DC-A9BA-7ABF77D8A2BB}" name="Content" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{8465D94C-DF8A-41D4-AE8E-1D443070FBA6}" name="Tableau730" displayName="Tableau730" ref="A12:C18" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{8465D94C-DF8A-41D4-AE8E-1D443070FBA6}" name="Tableau730" displayName="Tableau730" ref="A12:C18" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="A12:C18" xr:uid="{F9B6E3D6-4642-474A-BF1B-75555B5FB5E2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E70E637A-B135-4C05-9E37-8F59C5334F3F}" name="Benefit type" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{2C4F2AA3-1D7F-4D8D-9CC5-EE38E2406D17}" name="Amount" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{EBCC3121-CD73-4F5F-A831-498CDC42DCE6}" name="Details" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{E70E637A-B135-4C05-9E37-8F59C5334F3F}" name="Benefit type" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{2C4F2AA3-1D7F-4D8D-9CC5-EE38E2406D17}" name="Amount" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{EBCC3121-CD73-4F5F-A831-498CDC42DCE6}" name="Details" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{A94C271E-C976-4F7F-9940-CA8F0ED709CB}" name="Tableau1434" displayName="Tableau1434" ref="A3:C8" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{A94C271E-C976-4F7F-9940-CA8F0ED709CB}" name="Tableau1434" displayName="Tableau1434" ref="A3:C8" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A3:C8" xr:uid="{349C2764-B7C0-4860-B179-CA39241CFC68}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{8118D967-DD74-4ECE-9511-CF5E94FCDF24}" name="PSH Burkina Faso" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{E3AE2409-C96C-448C-9BB7-5F6E7AC835FD}" name="_x0009_Diesel Cost (LCOE)" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{396EBA3D-219C-4408-B208-797C91AB1F7B}" name="_x0009_Grid Emission Factor" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{8118D967-DD74-4ECE-9511-CF5E94FCDF24}" name="PSH Burkina Faso" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{E3AE2409-C96C-448C-9BB7-5F6E7AC835FD}" name="_x0009_Diesel Cost (LCOE)" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{396EBA3D-219C-4408-B208-797C91AB1F7B}" name="_x0009_Grid Emission Factor" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{1E764C27-A7D2-4E0E-AF6E-98984748B96C}" name="Tableau1131" displayName="Tableau1131" ref="A22:C25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{1E764C27-A7D2-4E0E-AF6E-98984748B96C}" name="Tableau1131" displayName="Tableau1131" ref="A22:C25" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A22:C25" xr:uid="{CED7CCD6-34C5-40BD-9E6D-857D4B0EDC6C}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{18D2097C-E6D3-4DA5-8D37-0FF753B15D00}" name="Benefit type" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{DBB759C5-F518-4E44-AF11-F4776C098EFB}" name="Amount" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{DB1CFD03-19DA-463E-8021-3A466300A71E}" name="Details" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{18D2097C-E6D3-4DA5-8D37-0FF753B15D00}" name="Benefit type" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{DBB759C5-F518-4E44-AF11-F4776C098EFB}" name="Amount" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{DB1CFD03-19DA-463E-8021-3A466300A71E}" name="Details" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{85116A30-0309-4BAF-8924-BDD017D62B49}" name="Table19" displayName="Table19" ref="A6:C14" totalsRowShown="0" headerRowDxfId="190" dataDxfId="189">
+  <autoFilter ref="A6:C14" xr:uid="{85116A30-0309-4BAF-8924-BDD017D62B49}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{DEB26626-8261-4F5A-A443-7D866F1D0938}" name="Parameter" dataDxfId="188"/>
+    <tableColumn id="2" xr3:uid="{39EFBE4A-9EFB-4CE8-BF1C-AEAC61E15A41}" name="Value" dataDxfId="187"/>
+    <tableColumn id="3" xr3:uid="{DC5FA7A1-A914-4FC1-8917-07FE7DE18DBA}" name="Source" dataDxfId="186"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{C220334E-603D-4753-B2EE-7AFDDC30B6C2}" name="Table20" displayName="Table20" ref="A21:F25" totalsRowShown="0" headerRowDxfId="185" dataDxfId="0">
+  <autoFilter ref="A21:F25" xr:uid="{C220334E-603D-4753-B2EE-7AFDDC30B6C2}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{7500FC79-9A77-4C8E-AF57-3BA27141CB47}" name="Scenario" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{BE3720ED-FE73-4092-BE3F-A5D903EF58A7}" name="Pump (corrected)" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{A663DFC8-DB81-4878-B9A8-131F6170187D}" name="Misc." dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{12722B78-C79F-4A50-B338-75D392C4BE71}" name="Extended (Aida)" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{2CD79A6F-F158-4E02-9A45-9C1AB21FC227}" name="Dryer" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{A84D8320-BE7E-4451-9647-8B339706B44A}" name="TOTAL (kWh/day)" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{BC6B92B9-47D8-49E1-AC47-78F5BBABBD66}" name="Table21" displayName="Table21" ref="A31:F35" totalsRowShown="0" headerRowDxfId="184" dataDxfId="183">
+  <autoFilter ref="A31:F35" xr:uid="{BC6B92B9-47D8-49E1-AC47-78F5BBABBD66}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{7D157030-B22C-4784-90A8-BA438D3C8811}" name="Scenario" dataDxfId="182"/>
+    <tableColumn id="2" xr3:uid="{3EBB14ED-A33C-4147-BEF1-A134A36EC264}" name="Energy (kWh/day)" dataDxfId="181"/>
+    <tableColumn id="3" xr3:uid="{0C3B211E-F279-417D-9C96-A60F192DB1B4}" name="PV required (kWp)" dataDxfId="180"/>
+    <tableColumn id="4" xr3:uid="{CFCB5658-EFB6-456B-BD54-994060C8AB3D}" name="No. of 400W panels" dataDxfId="179"/>
+    <tableColumn id="5" xr3:uid="{825B4CBD-A7EE-4484-9C58-FCD1AC3E9657}" name="Area (m²)" dataDxfId="178"/>
+    <tableColumn id="6" xr3:uid="{E00C9E3B-1E8E-4712-BA24-1EC8724903C8}" name="Area (ha)" dataDxfId="177"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{6BC8D30F-BA7E-4D9F-AD98-9FDECF2BE00D}" name="Table24" displayName="Table24" ref="A40:D44" totalsRowShown="0" headerRowDxfId="176" dataDxfId="175">
+  <autoFilter ref="A40:D44" xr:uid="{6BC8D30F-BA7E-4D9F-AD98-9FDECF2BE00D}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{95820E70-2839-4F38-B53F-D94EC6301DEF}" name="Scenario" dataDxfId="174"/>
+    <tableColumn id="2" xr3:uid="{96D3DC96-003C-4528-94E0-F493541A33A0}" name="Energy/8h (kWh)" dataDxfId="173"/>
+    <tableColumn id="3" xr3:uid="{675AD0AB-0540-4AA7-A28F-00112F40F97E}" name="With losses (kWh)" dataDxfId="172"/>
+    <tableColumn id="4" xr3:uid="{9D871537-E9CE-4692-9453-B87E1F626969}" name="Nominal capacity (kWh)" dataDxfId="171"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{1658F326-1A8F-4288-8B51-916A9592A7A3}" name="Table25" displayName="Table25" ref="A49:D53" totalsRowShown="0" headerRowDxfId="170" dataDxfId="7">
+  <autoFilter ref="A49:D53" xr:uid="{1658F326-1A8F-4288-8B51-916A9592A7A3}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{DFC44D2D-0577-4254-AC1E-2D257AE34515}" name="Scenario" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{D4EF2D05-833B-4958-AA7D-6EB222C04391}" name="PV cost ($)" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{17D5F8E1-89E0-4D52-ABD8-4D1C6D90A6C1}" name="Battery ($)" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{DB36AD43-0470-4B09-9243-78682D9A83F0}" name="Subtotal (excl. inverter)" dataDxfId="8"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{355CC7A6-D36C-4A5D-B23E-7CBB83FACBA8}" name="Table26" displayName="Table26" ref="A58:D64" totalsRowShown="0" headerRowDxfId="169" dataDxfId="12">
+  <autoFilter ref="A58:D64" xr:uid="{355CC7A6-D36C-4A5D-B23E-7CBB83FACBA8}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{A7B5702B-0434-446E-AE76-4FC9CC9828CF}" name="Parameter" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{9C68EE5C-4FB0-4C77-8E09-36E708F2CEC7}" name="Fixed-Tilt" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4A1FF7AA-E765-46CB-B309-B03E0210B3F5}" name="Tracking" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{B8273E41-3F1F-433A-B04B-FA596B4E5891}" name="Comment" dataDxfId="13"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4D45D2F0-98F4-43ED-A805-64E5D5307069}" name="Table6" displayName="Table6" ref="L26:Q30" totalsRowShown="0" headerRowDxfId="121" dataDxfId="120">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4D45D2F0-98F4-43ED-A805-64E5D5307069}" name="Table6" displayName="Table6" ref="L26:Q30" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149">
   <autoFilter ref="L26:Q30" xr:uid="{4D45D2F0-98F4-43ED-A805-64E5D5307069}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E184F488-E664-46EF-91BF-1BC45B8B521A}" name="Scenario" dataDxfId="119"/>
-    <tableColumn id="2" xr3:uid="{B98B6222-D44D-4BBF-B218-11D109C7445F}" name="Energy (kWh/day)" dataDxfId="118"/>
-    <tableColumn id="3" xr3:uid="{E5549AC5-ED05-4C8C-A6FA-381DDB3E6E9E}" name="PV required (kWp)" dataDxfId="117"/>
-    <tableColumn id="4" xr3:uid="{5DD47101-34B8-42BD-87ED-B1FB30E61E47}" name="No. of 400W panels" dataDxfId="116"/>
-    <tableColumn id="5" xr3:uid="{CFDEC47C-1CEF-47DC-8027-918F81A316DC}" name="Area (m²)" dataDxfId="115"/>
-    <tableColumn id="6" xr3:uid="{37A46260-E702-4679-BC93-FC760C77D1B8}" name="Area (ha)" dataDxfId="114"/>
+    <tableColumn id="1" xr3:uid="{E184F488-E664-46EF-91BF-1BC45B8B521A}" name="Scenario" dataDxfId="148"/>
+    <tableColumn id="2" xr3:uid="{B98B6222-D44D-4BBF-B218-11D109C7445F}" name="Energy (kWh/day)" dataDxfId="147"/>
+    <tableColumn id="3" xr3:uid="{E5549AC5-ED05-4C8C-A6FA-381DDB3E6E9E}" name="PV required (kWp)" dataDxfId="146"/>
+    <tableColumn id="4" xr3:uid="{5DD47101-34B8-42BD-87ED-B1FB30E61E47}" name="No. of 400W panels" dataDxfId="145"/>
+    <tableColumn id="5" xr3:uid="{CFDEC47C-1CEF-47DC-8027-918F81A316DC}" name="Area (m²)" dataDxfId="144"/>
+    <tableColumn id="6" xr3:uid="{37A46260-E702-4679-BC93-FC760C77D1B8}" name="Area (ha)" dataDxfId="143"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{6B08037B-52C5-49C0-8F6F-E6FE9C72F12C}" name="Table27" displayName="Table27" ref="A69:C74" totalsRowShown="0" headerRowDxfId="168" dataDxfId="167">
+  <autoFilter ref="A69:C74" xr:uid="{6B08037B-52C5-49C0-8F6F-E6FE9C72F12C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{37EF3812-ED85-4471-929C-0656BEFA852C}" name="Parameter" dataDxfId="166"/>
+    <tableColumn id="2" xr3:uid="{72DC59F3-7E8C-42D2-84A0-2A1471D3149A}" name="Value" dataDxfId="165"/>
+    <tableColumn id="3" xr3:uid="{3303A46E-8F97-42BC-AD15-F490BA867D57}" name="Comment" dataDxfId="164"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{D2D9C37A-6F72-49CE-898D-FC5F0CE19A37}" name="Table28" displayName="Table28" ref="A80:G84" totalsRowShown="0" headerRowDxfId="163" dataDxfId="21">
+  <autoFilter ref="A80:G84" xr:uid="{D2D9C37A-6F72-49CE-898D-FC5F0CE19A37}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{9B3BEAEB-38C2-41A1-88D5-145AE326479A}" name="Scenario" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{0A98C849-12D8-4FDA-9203-BF47220E7E98}" name="Annual Production (kWh/yr)" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{85F1816A-B173-44DE-8A1B-532118C47CC5}" name="PV Emissions (kg CO₂/yr)" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{D32CEF7F-479A-43F0-9832-5B6AC0562890}" name="Grid Equivalent (kg CO₂/yr)" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{27D5E875-5C7D-4F91-B51B-F6FF4D788E0B}" name="+ Generator" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{65796C6B-76F1-4087-B6E2-5019CBD5BB85}" name="Total Emissions" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{F2CE2B69-5242-4E63-AFD1-3DAA0F33EF68}" name="Reduction vs Grid" dataDxfId="22"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{AEE5F8D9-9F91-4123-9998-AD4F706B1F95}" name="Table29" displayName="Table29" ref="A89:C92" totalsRowShown="0" headerRowDxfId="162" dataDxfId="17">
+  <autoFilter ref="A89:C92" xr:uid="{AEE5F8D9-9F91-4123-9998-AD4F706B1F95}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{2ACDB6DF-C6C7-4D7B-A320-9FCBEA6A25B4}" name="Scenario" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{A326671F-F24E-4774-9DFF-B4100958271C}" name="Dried Output (kg/day)" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{ECD55F17-1929-4E9B-A30E-D38045028B0E}" name="CO₂/kg dried mango" dataDxfId="18"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{448951DC-D781-4A08-BE25-5788ACE67500}" name="Table7" displayName="Table7" ref="L35:O39" totalsRowShown="0" headerRowDxfId="113" dataDxfId="112">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{448951DC-D781-4A08-BE25-5788ACE67500}" name="Table7" displayName="Table7" ref="L35:O39" totalsRowShown="0" headerRowDxfId="142" dataDxfId="141">
   <autoFilter ref="L35:O39" xr:uid="{448951DC-D781-4A08-BE25-5788ACE67500}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{CD52C4E9-B061-4BC5-A1DB-9E5A4566A20C}" name="Scenario" dataDxfId="111"/>
-    <tableColumn id="2" xr3:uid="{C1A391E4-82E9-4B72-9009-5695DAE59118}" name="Energy/8h (kWh)" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{9CCF14E0-CA70-437A-9899-D47049433BE4}" name="With losses (kWh)" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{69FD8837-6441-4A3D-B0F7-A9468E6E3ECE}" name="Nominal capacity (kWh)" dataDxfId="108"/>
+    <tableColumn id="1" xr3:uid="{CD52C4E9-B061-4BC5-A1DB-9E5A4566A20C}" name="Scenario" dataDxfId="140"/>
+    <tableColumn id="2" xr3:uid="{C1A391E4-82E9-4B72-9009-5695DAE59118}" name="Energy/8h (kWh)" dataDxfId="139"/>
+    <tableColumn id="3" xr3:uid="{9CCF14E0-CA70-437A-9899-D47049433BE4}" name="With losses (kWh)" dataDxfId="138"/>
+    <tableColumn id="4" xr3:uid="{69FD8837-6441-4A3D-B0F7-A9468E6E3ECE}" name="Nominal capacity (kWh)" dataDxfId="137"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6A932467-02D2-4F2E-BE70-0C330E4A881D}" name="Table8" displayName="Table8" ref="L42:O46" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{6A932467-02D2-4F2E-BE70-0C330E4A881D}" name="Table8" displayName="Table8" ref="L42:O46" totalsRowShown="0" headerRowDxfId="136" dataDxfId="135">
   <autoFilter ref="L42:O46" xr:uid="{6A932467-02D2-4F2E-BE70-0C330E4A881D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{552D60E0-A25F-4E46-B279-FA5A28AA1063}" name="Scenario" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{642CE88C-057A-47CF-BF68-7A12CB200E13}" name="PV cost ($)" dataDxfId="104"/>
-    <tableColumn id="3" xr3:uid="{55087205-96A0-46B0-AC16-9EE825F3BD71}" name="Battery ($)" dataDxfId="103"/>
-    <tableColumn id="4" xr3:uid="{320CA687-C402-4CB2-8BF7-28D6D04E674B}" name="Subtotal (excl. inverter)" dataDxfId="102"/>
+    <tableColumn id="1" xr3:uid="{552D60E0-A25F-4E46-B279-FA5A28AA1063}" name="Scenario" dataDxfId="134"/>
+    <tableColumn id="2" xr3:uid="{642CE88C-057A-47CF-BF68-7A12CB200E13}" name="PV cost ($)" dataDxfId="133"/>
+    <tableColumn id="3" xr3:uid="{55087205-96A0-46B0-AC16-9EE825F3BD71}" name="Battery ($)" dataDxfId="132"/>
+    <tableColumn id="4" xr3:uid="{320CA687-C402-4CB2-8BF7-28D6D04E674B}" name="Subtotal (excl. inverter)" dataDxfId="131"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{10B49E62-8AA3-411B-B54C-2EE3F44D3D48}" name="Table9" displayName="Table9" ref="B68:C73" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{10B49E62-8AA3-411B-B54C-2EE3F44D3D48}" name="Table9" displayName="Table9" ref="B68:C73" totalsRowShown="0" headerRowDxfId="130" dataDxfId="129">
   <autoFilter ref="B68:C73" xr:uid="{10B49E62-8AA3-411B-B54C-2EE3F44D3D48}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{495A2024-60F6-42F7-981D-0EC286727055}" name="Screen" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{755049E7-3EEE-4DC5-B6B6-45D208956CBD}" name="Content" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{495A2024-60F6-42F7-981D-0EC286727055}" name="Screen" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{755049E7-3EEE-4DC5-B6B6-45D208956CBD}" name="Content" dataDxfId="127"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{D52F911D-F100-47D8-8FC3-5D3E0BD19D70}" name="Table10" displayName="Table10" ref="B58:D61" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{D52F911D-F100-47D8-8FC3-5D3E0BD19D70}" name="Table10" displayName="Table10" ref="B58:D61" totalsRowShown="0" headerRowDxfId="126" dataDxfId="125">
   <autoFilter ref="B58:D61" xr:uid="{D52F911D-F100-47D8-8FC3-5D3E0BD19D70}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CDDAE4F4-647F-46AB-8209-4530B35DD1FD}" name="Parameter" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{606BCBD9-AD3B-4A61-A962-F406C4A9C9E7}" name="Value" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{111B7450-F2A0-4F67-82FA-3C6C4767503A}" name="Comment" dataDxfId="93"/>
+    <tableColumn id="1" xr3:uid="{CDDAE4F4-647F-46AB-8209-4530B35DD1FD}" name="Parameter" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{606BCBD9-AD3B-4A61-A962-F406C4A9C9E7}" name="Value" dataDxfId="123"/>
+    <tableColumn id="3" xr3:uid="{111B7450-F2A0-4F67-82FA-3C6C4767503A}" name="Comment" dataDxfId="122"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{7644C370-D105-445A-8279-9ECADCBE6A9E}" name="Table11" displayName="Table11" ref="F58:L62" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{7644C370-D105-445A-8279-9ECADCBE6A9E}" name="Table11" displayName="Table11" ref="F58:L62" totalsRowShown="0" headerRowDxfId="121" dataDxfId="120">
   <autoFilter ref="F58:L62" xr:uid="{7644C370-D105-445A-8279-9ECADCBE6A9E}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{61CB783B-62C3-4E8F-8575-BC96FEDAF728}" name="Scenario" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{79394F7B-B735-4C81-8FBE-1486C4434AC3}" name="Annual Production (kWh/yr)" dataDxfId="89"/>
-    <tableColumn id="3" xr3:uid="{18962A85-CC51-4E5E-83E0-8A13A08C4E62}" name="PV Emissions (kg CO₂/yr)" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{865B7B3E-A775-4B4B-8663-EC6EC3DABC68}" name="Grid Equivalent (kg CO₂/yr)" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{C4FB733B-8D99-459A-A5AF-2972523D20CC}" name="+ Generator (kg CO₂/yr)" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{516A31C3-73B9-4402-AD5F-F059B6FC291A}" name="Total System Emissions" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{9791C282-DAF0-47EE-8AA7-3236043798C0}" name="Reduction vs Grid" dataDxfId="84"/>
+    <tableColumn id="1" xr3:uid="{61CB783B-62C3-4E8F-8575-BC96FEDAF728}" name="Scenario" dataDxfId="119"/>
+    <tableColumn id="2" xr3:uid="{79394F7B-B735-4C81-8FBE-1486C4434AC3}" name="Annual Production (kWh/yr)" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{18962A85-CC51-4E5E-83E0-8A13A08C4E62}" name="PV Emissions (kg CO₂/yr)" dataDxfId="117"/>
+    <tableColumn id="4" xr3:uid="{865B7B3E-A775-4B4B-8663-EC6EC3DABC68}" name="Grid Equivalent (kg CO₂/yr)" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{C4FB733B-8D99-459A-A5AF-2972523D20CC}" name="+ Generator (kg CO₂/yr)" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{516A31C3-73B9-4402-AD5F-F059B6FC291A}" name="Total System Emissions" dataDxfId="114"/>
+    <tableColumn id="7" xr3:uid="{9791C282-DAF0-47EE-8AA7-3236043798C0}" name="Reduction vs Grid" dataDxfId="113"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B3B5BED7-8BB6-49C3-B05F-F5D5322B309C}" name="Table12" displayName="Table12" ref="B5:C16" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B3B5BED7-8BB6-49C3-B05F-F5D5322B309C}" name="Table12" displayName="Table12" ref="B5:C16" totalsRowShown="0" headerRowDxfId="112" dataDxfId="111">
   <autoFilter ref="B5:C16" xr:uid="{B3B5BED7-8BB6-49C3-B05F-F5D5322B309C}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0CC8CD02-1550-4F7E-B71E-A56A49340243}" name="Term / Abbreviation" dataDxfId="81"/>
-    <tableColumn id="2" xr3:uid="{97DCE0BE-9ACE-4F27-8A8B-7240E5BB77F3}" name="Definition" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{0CC8CD02-1550-4F7E-B71E-A56A49340243}" name="Term / Abbreviation" dataDxfId="110"/>
+    <tableColumn id="2" xr3:uid="{97DCE0BE-9ACE-4F27-8A8B-7240E5BB77F3}" name="Definition" dataDxfId="109"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5316,30 +6912,30 @@
       <c r="K1" s="26"/>
     </row>
     <row r="2" spans="2:19" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="137" t="s">
+      <c r="B2" s="130" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="138"/>
+      <c r="C2" s="131"/>
       <c r="D2" s="29"/>
-      <c r="E2" s="139" t="s">
+      <c r="E2" s="132" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="140"/>
-      <c r="G2" s="141"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="134"/>
       <c r="H2" s="29"/>
-      <c r="I2" s="144" t="s">
+      <c r="I2" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="145"/>
-      <c r="K2" s="145"/>
-      <c r="L2" s="145"/>
-      <c r="M2" s="146"/>
-      <c r="P2" s="128" t="s">
+      <c r="J2" s="138"/>
+      <c r="K2" s="138"/>
+      <c r="L2" s="138"/>
+      <c r="M2" s="139"/>
+      <c r="P2" s="121" t="s">
         <v>317</v>
       </c>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
+      <c r="Q2" s="122"/>
+      <c r="R2" s="122"/>
+      <c r="S2" s="122"/>
     </row>
     <row r="3" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B3" s="82" t="s">
@@ -5479,7 +7075,7 @@
         <v>182.5</v>
       </c>
     </row>
-    <row r="6" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B6" s="33" t="s">
         <v>48</v>
       </c>
@@ -5525,7 +7121,7 @@
         <v>632.5</v>
       </c>
     </row>
-    <row r="7" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B7" s="33" t="s">
         <v>12</v>
       </c>
@@ -5571,7 +7167,7 @@
         <v>3032.5</v>
       </c>
     </row>
-    <row r="8" spans="2:19" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.3">
       <c r="B8" s="33" t="s">
         <v>13</v>
       </c>
@@ -5598,15 +7194,15 @@
       <c r="C9" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="142" t="s">
+      <c r="E9" s="135" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="143"/>
-      <c r="H9" s="131" t="s">
+      <c r="F9" s="136"/>
+      <c r="H9" s="124" t="s">
         <v>303</v>
       </c>
-      <c r="I9" s="132"/>
-      <c r="J9" s="132"/>
+      <c r="I9" s="125"/>
+      <c r="J9" s="125"/>
       <c r="K9" s="32"/>
       <c r="L9" s="5"/>
     </row>
@@ -5777,15 +7373,15 @@
       <c r="R15" s="32"/>
     </row>
     <row r="16" spans="2:19" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="147" t="s">
+      <c r="B16" s="140" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="147"/>
-      <c r="D16" s="147"/>
-      <c r="F16" s="148" t="s">
+      <c r="C16" s="140"/>
+      <c r="D16" s="140"/>
+      <c r="F16" s="141" t="s">
         <v>76</v>
       </c>
-      <c r="G16" s="148"/>
+      <c r="G16" s="141"/>
       <c r="H16" s="37"/>
       <c r="O16" s="31"/>
       <c r="P16" s="31"/>
@@ -5928,26 +7524,26 @@
       <c r="L24" s="5"/>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B25" s="136" t="s">
+      <c r="B25" s="129" t="s">
         <v>92</v>
       </c>
-      <c r="C25" s="136"/>
-      <c r="D25" s="136"/>
-      <c r="E25" s="136"/>
-      <c r="F25" s="136"/>
-      <c r="G25" s="136"/>
-      <c r="H25" s="136"/>
-      <c r="I25" s="136"/>
-      <c r="J25" s="136"/>
+      <c r="C25" s="129"/>
+      <c r="D25" s="129"/>
+      <c r="E25" s="129"/>
+      <c r="F25" s="129"/>
+      <c r="G25" s="129"/>
+      <c r="H25" s="129"/>
+      <c r="I25" s="129"/>
+      <c r="J25" s="129"/>
       <c r="K25" s="44"/>
-      <c r="L25" s="130" t="s">
+      <c r="L25" s="123" t="s">
         <v>321</v>
       </c>
-      <c r="M25" s="130"/>
-      <c r="N25" s="130"/>
-      <c r="O25" s="130"/>
-      <c r="P25" s="130"/>
-      <c r="Q25" s="130"/>
+      <c r="M25" s="123"/>
+      <c r="N25" s="123"/>
+      <c r="O25" s="123"/>
+      <c r="P25" s="123"/>
+      <c r="Q25" s="123"/>
     </row>
     <row r="26" spans="2:18" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B26" s="81" t="s">
@@ -6175,15 +7771,15 @@
       <c r="L32" s="5"/>
     </row>
     <row r="33" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B33" s="133" t="s">
+      <c r="B33" s="126" t="s">
         <v>99</v>
       </c>
-      <c r="C33" s="133"/>
-      <c r="D33" s="133"/>
-      <c r="E33" s="133"/>
-      <c r="F33" s="133"/>
-      <c r="G33" s="133"/>
-      <c r="H33" s="133"/>
+      <c r="C33" s="126"/>
+      <c r="D33" s="126"/>
+      <c r="E33" s="126"/>
+      <c r="F33" s="126"/>
+      <c r="G33" s="126"/>
+      <c r="H33" s="126"/>
       <c r="J33" s="45"/>
       <c r="K33" s="45"/>
       <c r="N33"/>
@@ -6358,16 +7954,16 @@
       </c>
     </row>
     <row r="40" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B40" s="134" t="s">
+      <c r="B40" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="C40" s="134"/>
-      <c r="D40" s="134"/>
-      <c r="E40" s="134"/>
-      <c r="F40" s="134"/>
-      <c r="G40" s="134"/>
-      <c r="H40" s="134"/>
-      <c r="I40" s="134"/>
+      <c r="C40" s="127"/>
+      <c r="D40" s="127"/>
+      <c r="E40" s="127"/>
+      <c r="F40" s="127"/>
+      <c r="G40" s="127"/>
+      <c r="H40" s="127"/>
+      <c r="I40" s="127"/>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="81" t="s">
@@ -6392,12 +7988,12 @@
       <c r="I41" s="81" t="s">
         <v>115</v>
       </c>
-      <c r="L41" s="131" t="s">
+      <c r="L41" s="124" t="s">
         <v>326</v>
       </c>
-      <c r="M41" s="131"/>
-      <c r="N41" s="131"/>
-      <c r="O41" s="131"/>
+      <c r="M41" s="124"/>
+      <c r="N41" s="124"/>
+      <c r="O41" s="124"/>
     </row>
     <row r="42" spans="2:15" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B42" s="30" t="s">
@@ -6568,17 +8164,17 @@
       <c r="G47" s="52"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B48" s="135" t="s">
+      <c r="B48" s="128" t="s">
         <v>122</v>
       </c>
-      <c r="C48" s="135"/>
-      <c r="D48" s="135"/>
-      <c r="E48" s="135"/>
-      <c r="F48" s="135"/>
-      <c r="G48" s="135"/>
-      <c r="H48" s="135"/>
-      <c r="I48" s="135"/>
-      <c r="J48" s="135"/>
+      <c r="C48" s="128"/>
+      <c r="D48" s="128"/>
+      <c r="E48" s="128"/>
+      <c r="F48" s="128"/>
+      <c r="G48" s="128"/>
+      <c r="H48" s="128"/>
+      <c r="I48" s="128"/>
+      <c r="J48" s="128"/>
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="81" t="s">
@@ -6727,19 +8323,19 @@
       <c r="G55" s="57"/>
     </row>
     <row r="56" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B56" s="131" t="s">
+      <c r="B56" s="124" t="s">
         <v>328</v>
       </c>
-      <c r="C56" s="132"/>
-      <c r="D56" s="132"/>
-      <c r="E56" s="132"/>
-      <c r="F56" s="132"/>
-      <c r="G56" s="132"/>
-      <c r="H56" s="132"/>
-      <c r="I56" s="132"/>
-      <c r="J56" s="132"/>
-      <c r="K56" s="132"/>
-      <c r="L56" s="132"/>
+      <c r="C56" s="125"/>
+      <c r="D56" s="125"/>
+      <c r="E56" s="125"/>
+      <c r="F56" s="125"/>
+      <c r="G56" s="125"/>
+      <c r="H56" s="125"/>
+      <c r="I56" s="125"/>
+      <c r="J56" s="125"/>
+      <c r="K56" s="125"/>
+      <c r="L56" s="125"/>
     </row>
     <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="57"/>
@@ -6932,10 +8528,10 @@
       <c r="G65" s="65"/>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B66" s="127" t="s">
+      <c r="B66" s="120" t="s">
         <v>343</v>
       </c>
-      <c r="C66" s="127"/>
+      <c r="C66" s="120"/>
       <c r="D66"/>
       <c r="E66" s="67"/>
       <c r="F66" s="67"/>
@@ -7128,10 +8724,10 @@
     </row>
     <row r="7" spans="6:11" ht="18" x14ac:dyDescent="0.35">
       <c r="F7" s="88"/>
-      <c r="G7" s="121" t="s">
+      <c r="G7" s="119" t="s">
         <v>265</v>
       </c>
-      <c r="H7" s="120"/>
+      <c r="H7" s="144"/>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="6:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -7262,10 +8858,10 @@
     </row>
     <row r="19" spans="6:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="F19" s="88"/>
-      <c r="G19" s="118" t="s">
+      <c r="G19" s="142" t="s">
         <v>264</v>
       </c>
-      <c r="H19" s="120"/>
+      <c r="H19" s="144"/>
       <c r="I19" s="88"/>
     </row>
     <row r="20" spans="6:9" ht="18" x14ac:dyDescent="0.35">
@@ -7442,10 +9038,10 @@
     </row>
     <row r="34" spans="6:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="F34" s="19"/>
-      <c r="G34" s="125" t="s">
+      <c r="G34" s="148" t="s">
         <v>263</v>
       </c>
-      <c r="H34" s="126"/>
+      <c r="H34" s="149"/>
       <c r="I34" s="88"/>
     </row>
     <row r="35" spans="6:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -7581,10 +9177,10 @@
     </row>
     <row r="45" spans="6:10" ht="21" x14ac:dyDescent="0.4">
       <c r="F45" s="18"/>
-      <c r="G45" s="123" t="s">
+      <c r="G45" s="146" t="s">
         <v>262</v>
       </c>
-      <c r="H45" s="124"/>
+      <c r="H45" s="147"/>
       <c r="I45" s="18"/>
       <c r="J45" s="4"/>
     </row>
@@ -7676,10 +9272,10 @@
     </row>
     <row r="53" spans="6:10" ht="21" x14ac:dyDescent="0.4">
       <c r="F53" s="3"/>
-      <c r="G53" s="118" t="s">
+      <c r="G53" s="142" t="s">
         <v>261</v>
       </c>
-      <c r="H53" s="122"/>
+      <c r="H53" s="145"/>
       <c r="I53" s="3"/>
       <c r="J53" s="3"/>
     </row>
@@ -7855,10 +9451,10 @@
     </row>
     <row r="67" spans="6:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F67" s="8"/>
-      <c r="G67" s="121" t="s">
+      <c r="G67" s="119" t="s">
         <v>260</v>
       </c>
-      <c r="H67" s="120"/>
+      <c r="H67" s="144"/>
       <c r="I67" s="6"/>
     </row>
     <row r="68" spans="6:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -7979,10 +9575,10 @@
     </row>
     <row r="78" spans="6:9" ht="18" x14ac:dyDescent="0.35">
       <c r="F78" s="6"/>
-      <c r="G78" s="121" t="s">
+      <c r="G78" s="119" t="s">
         <v>259</v>
       </c>
-      <c r="H78" s="120"/>
+      <c r="H78" s="144"/>
       <c r="I78" s="6"/>
     </row>
     <row r="79" spans="6:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -8042,10 +9638,10 @@
       </c>
     </row>
     <row r="86" spans="6:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="G86" s="118" t="s">
+      <c r="G86" s="142" t="s">
         <v>257</v>
       </c>
-      <c r="H86" s="119"/>
+      <c r="H86" s="143"/>
     </row>
     <row r="88" spans="6:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="F88" s="91" t="s">
@@ -8488,10 +10084,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:27" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="131" t="s">
+      <c r="B4" s="124" t="s">
         <v>350</v>
       </c>
-      <c r="C4" s="132"/>
+      <c r="C4" s="125"/>
     </row>
     <row r="5" spans="2:27" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="96" t="s">
@@ -8509,31 +10105,31 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="2:27" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:27" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B7" s="97" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="97" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="131" t="s">
+      <c r="L7" s="124" t="s">
         <v>352</v>
       </c>
-      <c r="M7" s="131"/>
-      <c r="N7" s="131"/>
-      <c r="R7" s="131" t="s">
+      <c r="M7" s="124"/>
+      <c r="N7" s="124"/>
+      <c r="R7" s="124" t="s">
         <v>353</v>
       </c>
-      <c r="S7" s="132"/>
-      <c r="T7" s="132"/>
-      <c r="X7" s="128" t="s">
+      <c r="S7" s="125"/>
+      <c r="T7" s="125"/>
+      <c r="X7" s="121" t="s">
         <v>317</v>
       </c>
-      <c r="Y7" s="129"/>
-      <c r="Z7" s="129"/>
-      <c r="AA7" s="129"/>
-    </row>
-    <row r="8" spans="2:27" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="Y7" s="122"/>
+      <c r="Z7" s="122"/>
+      <c r="AA7" s="122"/>
+    </row>
+    <row r="8" spans="2:27" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B8" s="97" t="s">
         <v>48</v>
       </c>
@@ -8753,10 +10349,10 @@
       <c r="C15" s="97" t="s">
         <v>70</v>
       </c>
-      <c r="L15" s="155" t="s">
+      <c r="L15" s="156" t="s">
         <v>354</v>
       </c>
-      <c r="M15" s="143"/>
+      <c r="M15" s="136"/>
     </row>
     <row r="16" spans="2:27" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B16" s="97" t="s">
@@ -8772,7 +10368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="2:13" ht="62.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="L17" s="30" t="s">
         <v>64</v>
       </c>
@@ -8805,11 +10401,11 @@
       </c>
     </row>
     <row r="22" spans="2:13" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="147" t="s">
+      <c r="B22" s="140" t="s">
         <v>355</v>
       </c>
-      <c r="C22" s="147"/>
-      <c r="D22" s="147"/>
+      <c r="C22" s="140"/>
+      <c r="D22" s="140"/>
     </row>
     <row r="23" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B23" s="82" t="s">
@@ -8821,10 +10417,10 @@
       <c r="D23" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="L23" s="148" t="s">
+      <c r="L23" s="141" t="s">
         <v>356</v>
       </c>
-      <c r="M23" s="148"/>
+      <c r="M23" s="141"/>
     </row>
     <row r="24" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B24" s="33" t="s">
@@ -8913,17 +10509,17 @@
       </c>
     </row>
     <row r="33" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B33" s="136" t="s">
+      <c r="B33" s="129" t="s">
         <v>92</v>
       </c>
-      <c r="C33" s="136"/>
-      <c r="D33" s="136"/>
-      <c r="E33" s="136"/>
-      <c r="F33" s="136"/>
-      <c r="G33" s="136"/>
-      <c r="H33" s="136"/>
-      <c r="I33" s="136"/>
-      <c r="J33" s="136"/>
+      <c r="C33" s="129"/>
+      <c r="D33" s="129"/>
+      <c r="E33" s="129"/>
+      <c r="F33" s="129"/>
+      <c r="G33" s="129"/>
+      <c r="H33" s="129"/>
+      <c r="I33" s="129"/>
+      <c r="J33" s="129"/>
     </row>
     <row r="35" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B35" s="81" t="s">
@@ -8932,14 +10528,14 @@
       <c r="C35" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="130" t="s">
+      <c r="E35" s="123" t="s">
         <v>321</v>
       </c>
-      <c r="F35" s="130"/>
-      <c r="G35" s="130"/>
-      <c r="H35" s="130"/>
-      <c r="I35" s="130"/>
-      <c r="J35" s="130"/>
+      <c r="F35" s="123"/>
+      <c r="G35" s="123"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="123"/>
+      <c r="J35" s="123"/>
     </row>
     <row r="36" spans="2:10" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B36" s="30" t="s">
@@ -8987,7 +10583,7 @@
         <v>5.5999999999999999E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E38" s="97" t="s">
         <v>47</v>
       </c>
@@ -9007,7 +10603,7 @@
         <v>3.1300000000000001E-2</v>
       </c>
     </row>
-    <row r="39" spans="2:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E39" s="97" t="s">
         <v>53</v>
       </c>
@@ -9027,7 +10623,7 @@
         <v>0.1086</v>
       </c>
     </row>
-    <row r="40" spans="2:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E40" s="97" t="s">
         <v>58</v>
       </c>
@@ -9048,17 +10644,17 @@
       </c>
     </row>
     <row r="44" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B44" s="153" t="s">
+      <c r="B44" s="154" t="s">
         <v>99</v>
       </c>
-      <c r="C44" s="154"/>
-      <c r="D44" s="154"/>
-      <c r="E44" s="154"/>
-      <c r="F44" s="154"/>
-      <c r="G44" s="154"/>
-      <c r="H44" s="154"/>
-      <c r="I44" s="154"/>
-      <c r="J44" s="154"/>
+      <c r="C44" s="155"/>
+      <c r="D44" s="155"/>
+      <c r="E44" s="155"/>
+      <c r="F44" s="155"/>
+      <c r="G44" s="155"/>
+      <c r="H44" s="155"/>
+      <c r="I44" s="155"/>
+      <c r="J44" s="155"/>
     </row>
     <row r="46" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B46" s="82" t="s">
@@ -9163,16 +10759,16 @@
       </c>
     </row>
     <row r="55" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B55" s="134" t="s">
+      <c r="B55" s="127" t="s">
         <v>109</v>
       </c>
-      <c r="C55" s="134"/>
-      <c r="D55" s="134"/>
-      <c r="E55" s="134"/>
-      <c r="F55" s="134"/>
-      <c r="G55" s="134"/>
-      <c r="H55" s="134"/>
-      <c r="I55" s="134"/>
+      <c r="C55" s="127"/>
+      <c r="D55" s="127"/>
+      <c r="E55" s="127"/>
+      <c r="F55" s="127"/>
+      <c r="G55" s="127"/>
+      <c r="H55" s="127"/>
+      <c r="I55" s="127"/>
     </row>
     <row r="57" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B57" s="81" t="s">
@@ -9181,12 +10777,12 @@
       <c r="C57" s="81" t="s">
         <v>111</v>
       </c>
-      <c r="F57" s="131" t="s">
+      <c r="F57" s="124" t="s">
         <v>326</v>
       </c>
-      <c r="G57" s="131"/>
-      <c r="H57" s="131"/>
-      <c r="I57" s="131"/>
+      <c r="G57" s="124"/>
+      <c r="H57" s="124"/>
+      <c r="I57" s="124"/>
     </row>
     <row r="58" spans="2:9" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B58" s="30" t="s">
@@ -9277,16 +10873,16 @@
       </c>
     </row>
     <row r="67" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B67" s="151" t="s">
+      <c r="B67" s="152" t="s">
         <v>357</v>
       </c>
-      <c r="C67" s="134"/>
-      <c r="D67" s="134"/>
-      <c r="E67" s="134"/>
-      <c r="F67" s="134"/>
-      <c r="G67" s="134"/>
-      <c r="H67" s="134"/>
-      <c r="I67" s="134"/>
+      <c r="C67" s="127"/>
+      <c r="D67" s="127"/>
+      <c r="E67" s="127"/>
+      <c r="F67" s="127"/>
+      <c r="G67" s="127"/>
+      <c r="H67" s="127"/>
+      <c r="I67" s="127"/>
     </row>
     <row r="69" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B69" s="96" t="s">
@@ -9316,7 +10912,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="71" spans="2:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B71" s="97" t="s">
         <v>363</v>
       </c>
@@ -9359,16 +10955,16 @@
       </c>
     </row>
     <row r="76" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B76" s="152" t="s">
+      <c r="B76" s="153" t="s">
         <v>368</v>
       </c>
-      <c r="C76" s="134"/>
-      <c r="D76" s="134"/>
-      <c r="E76" s="134"/>
-      <c r="F76" s="134"/>
-      <c r="G76" s="134"/>
-      <c r="H76" s="134"/>
-      <c r="I76" s="134"/>
+      <c r="C76" s="127"/>
+      <c r="D76" s="127"/>
+      <c r="E76" s="127"/>
+      <c r="F76" s="127"/>
+      <c r="G76" s="127"/>
+      <c r="H76" s="127"/>
+      <c r="I76" s="127"/>
     </row>
     <row r="78" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B78" s="96" t="s">
@@ -9381,7 +10977,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="2:9" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:9" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B79" s="97" t="s">
         <v>369</v>
       </c>
@@ -9414,7 +11010,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="82" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B82" s="97" t="s">
         <v>273</v>
       </c>
@@ -9469,7 +11065,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="87" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B87" s="97" t="s">
         <v>384</v>
       </c>
@@ -9481,19 +11077,19 @@
       </c>
     </row>
     <row r="90" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B90" s="149" t="s">
+      <c r="B90" s="150" t="s">
         <v>387</v>
       </c>
-      <c r="C90" s="150"/>
-      <c r="D90" s="150"/>
-      <c r="E90" s="150"/>
-      <c r="F90" s="150"/>
-      <c r="G90" s="150"/>
-      <c r="H90" s="150"/>
-      <c r="I90" s="150"/>
-      <c r="J90" s="150"/>
-      <c r="K90" s="150"/>
-      <c r="L90" s="150"/>
+      <c r="C90" s="151"/>
+      <c r="D90" s="151"/>
+      <c r="E90" s="151"/>
+      <c r="F90" s="151"/>
+      <c r="G90" s="151"/>
+      <c r="H90" s="151"/>
+      <c r="I90" s="151"/>
+      <c r="J90" s="151"/>
+      <c r="K90" s="151"/>
+      <c r="L90" s="151"/>
     </row>
     <row r="92" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B92" s="96" t="s">
@@ -9647,19 +11243,19 @@
       </c>
     </row>
     <row r="100" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B100" s="149" t="s">
+      <c r="B100" s="150" t="s">
         <v>388</v>
       </c>
-      <c r="C100" s="150"/>
-      <c r="D100" s="150"/>
-      <c r="E100" s="150"/>
-      <c r="F100" s="150"/>
-      <c r="G100" s="150"/>
-      <c r="H100" s="150"/>
-      <c r="I100" s="150"/>
-      <c r="J100" s="150"/>
-      <c r="K100" s="150"/>
-      <c r="L100" s="150"/>
+      <c r="C100" s="151"/>
+      <c r="D100" s="151"/>
+      <c r="E100" s="151"/>
+      <c r="F100" s="151"/>
+      <c r="G100" s="151"/>
+      <c r="H100" s="151"/>
+      <c r="I100" s="151"/>
+      <c r="J100" s="151"/>
+      <c r="K100" s="151"/>
+      <c r="L100" s="151"/>
     </row>
     <row r="101" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B101" s="96" t="s">
@@ -9669,7 +11265,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="102" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B102" s="97" t="s">
         <v>292</v>
       </c>
@@ -9677,7 +11273,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="103" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:12" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B103" s="97" t="s">
         <v>294</v>
       </c>
@@ -9685,7 +11281,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="104" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B104" s="97" t="s">
         <v>296</v>
       </c>
@@ -9693,7 +11289,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="105" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B105" s="97" t="s">
         <v>298</v>
       </c>
@@ -9701,7 +11297,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="106" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B106" s="97" t="s">
         <v>300</v>
       </c>
@@ -9804,28 +11400,28 @@
       <c r="C7" s="112"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="156"/>
-      <c r="C9" s="156"/>
-      <c r="D9" s="156"/>
-      <c r="E9" s="156"/>
-      <c r="F9" s="156"/>
+      <c r="B9" s="118"/>
+      <c r="C9" s="118"/>
+      <c r="D9" s="118"/>
+      <c r="E9" s="118"/>
+      <c r="F9" s="118"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="110" t="s">
         <v>395</v>
       </c>
-      <c r="B10" s="156"/>
-      <c r="C10" s="156"/>
-      <c r="D10" s="156"/>
-      <c r="E10" s="156"/>
-      <c r="F10" s="156"/>
+      <c r="B10" s="118"/>
+      <c r="C10" s="118"/>
+      <c r="D10" s="118"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="118"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="156"/>
-      <c r="C11" s="156"/>
-      <c r="D11" s="156"/>
-      <c r="E11" s="156"/>
-      <c r="F11" s="156"/>
+      <c r="B11" s="118"/>
+      <c r="C11" s="118"/>
+      <c r="D11" s="118"/>
+      <c r="E11" s="118"/>
+      <c r="F11" s="118"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="93" t="s">
@@ -9895,28 +11491,28 @@
       <c r="A18" s="111"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B19" s="156"/>
-      <c r="C19" s="156"/>
-      <c r="D19" s="156"/>
-      <c r="E19" s="156"/>
-      <c r="F19" s="156"/>
+      <c r="B19" s="118"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="110" t="s">
         <v>412</v>
       </c>
-      <c r="B20" s="156"/>
-      <c r="C20" s="156"/>
-      <c r="D20" s="156"/>
-      <c r="E20" s="156"/>
-      <c r="F20" s="156"/>
+      <c r="B20" s="118"/>
+      <c r="C20" s="118"/>
+      <c r="D20" s="118"/>
+      <c r="E20" s="118"/>
+      <c r="F20" s="118"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B21" s="156"/>
-      <c r="C21" s="156"/>
-      <c r="D21" s="156"/>
-      <c r="E21" s="156"/>
-      <c r="F21" s="156"/>
+      <c r="B21" s="118"/>
+      <c r="C21" s="118"/>
+      <c r="D21" s="118"/>
+      <c r="E21" s="118"/>
+      <c r="F21" s="118"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="93" t="s">
@@ -10070,4 +11666,873 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B7C1208-BF31-4EDF-9156-8741784C1003}">
+  <dimension ref="A4:G92"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.6640625" style="107" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" style="107" customWidth="1"/>
+    <col min="3" max="3" width="31.109375" style="107" customWidth="1"/>
+    <col min="4" max="4" width="33.88671875" style="107" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" style="107" customWidth="1"/>
+    <col min="6" max="6" width="24" style="107" customWidth="1"/>
+    <col min="7" max="7" width="23" style="107" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="107"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="118" t="s">
+        <v>303</v>
+      </c>
+      <c r="B4" s="118"/>
+      <c r="C4" s="118"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="93" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="93" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="93" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="94" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="94" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="94" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="52.2" x14ac:dyDescent="0.35">
+      <c r="A8" s="115" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="115" t="s">
+        <v>505</v>
+      </c>
+      <c r="C8" s="115" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="36" x14ac:dyDescent="0.35">
+      <c r="A9" s="94" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="94" t="s">
+        <v>427</v>
+      </c>
+      <c r="C9" s="94" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="94" t="s">
+        <v>177</v>
+      </c>
+      <c r="B10" s="94" t="s">
+        <v>304</v>
+      </c>
+      <c r="C10" s="94" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="94" t="s">
+        <v>305</v>
+      </c>
+      <c r="B11" s="94" t="s">
+        <v>306</v>
+      </c>
+      <c r="C11" s="94" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="36" x14ac:dyDescent="0.35">
+      <c r="A12" s="94" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" s="94" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" s="94" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="94" t="s">
+        <v>309</v>
+      </c>
+      <c r="B13" s="94" t="s">
+        <v>310</v>
+      </c>
+      <c r="C13" s="94" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="34.799999999999997" x14ac:dyDescent="0.35">
+      <c r="A14" s="115" t="s">
+        <v>351</v>
+      </c>
+      <c r="B14" s="115" t="s">
+        <v>316</v>
+      </c>
+      <c r="C14" s="94"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="118" t="s">
+        <v>430</v>
+      </c>
+      <c r="B19" s="118"/>
+      <c r="C19" s="118"/>
+      <c r="D19" s="118"/>
+      <c r="E19" s="118"/>
+      <c r="F19" s="118"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="C21" s="93" t="s">
+        <v>431</v>
+      </c>
+      <c r="D21" s="93" t="s">
+        <v>432</v>
+      </c>
+      <c r="E21" s="93" t="s">
+        <v>5</v>
+      </c>
+      <c r="F21" s="93" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="116" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="159" t="s">
+        <v>433</v>
+      </c>
+      <c r="C22" s="116">
+        <v>15</v>
+      </c>
+      <c r="D22" s="116" t="s">
+        <v>434</v>
+      </c>
+      <c r="E22" s="116">
+        <v>0</v>
+      </c>
+      <c r="F22" s="159" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="116" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="159" t="s">
+        <v>433</v>
+      </c>
+      <c r="C23" s="116">
+        <v>15</v>
+      </c>
+      <c r="D23" s="116" t="s">
+        <v>434</v>
+      </c>
+      <c r="E23" s="116">
+        <v>150</v>
+      </c>
+      <c r="F23" s="159" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="116" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="159" t="s">
+        <v>433</v>
+      </c>
+      <c r="C24" s="116">
+        <v>15</v>
+      </c>
+      <c r="D24" s="116" t="s">
+        <v>434</v>
+      </c>
+      <c r="E24" s="116">
+        <v>600</v>
+      </c>
+      <c r="F24" s="159" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="116" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="159" t="s">
+        <v>433</v>
+      </c>
+      <c r="C25" s="116">
+        <v>15</v>
+      </c>
+      <c r="D25" s="116" t="s">
+        <v>434</v>
+      </c>
+      <c r="E25" s="116">
+        <v>3</v>
+      </c>
+      <c r="F25" s="159" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="118" t="s">
+        <v>439</v>
+      </c>
+      <c r="B28" s="118"/>
+      <c r="C28" s="118"/>
+      <c r="D28" s="118"/>
+      <c r="E28" s="118"/>
+      <c r="F28" s="118"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="93" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="93" t="s">
+        <v>93</v>
+      </c>
+      <c r="D31" s="93" t="s">
+        <v>94</v>
+      </c>
+      <c r="E31" s="93" t="s">
+        <v>322</v>
+      </c>
+      <c r="F31" s="93" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="94" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="94" t="s">
+        <v>435</v>
+      </c>
+      <c r="C32" s="94" t="s">
+        <v>440</v>
+      </c>
+      <c r="D32" s="94">
+        <v>18</v>
+      </c>
+      <c r="E32" s="94" t="s">
+        <v>441</v>
+      </c>
+      <c r="F32" s="94" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="94" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="94" t="s">
+        <v>436</v>
+      </c>
+      <c r="C33" s="94" t="s">
+        <v>443</v>
+      </c>
+      <c r="D33" s="94">
+        <v>93</v>
+      </c>
+      <c r="E33" s="94" t="s">
+        <v>444</v>
+      </c>
+      <c r="F33" s="94" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="94" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="94" t="s">
+        <v>437</v>
+      </c>
+      <c r="C34" s="94" t="s">
+        <v>446</v>
+      </c>
+      <c r="D34" s="94">
+        <v>321</v>
+      </c>
+      <c r="E34" s="94" t="s">
+        <v>447</v>
+      </c>
+      <c r="F34" s="94" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="94" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="94" t="s">
+        <v>438</v>
+      </c>
+      <c r="C35" s="94" t="s">
+        <v>449</v>
+      </c>
+      <c r="D35" s="94">
+        <v>1.5329999999999999</v>
+      </c>
+      <c r="E35" s="94" t="s">
+        <v>450</v>
+      </c>
+      <c r="F35" s="94" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="118" t="s">
+        <v>452</v>
+      </c>
+      <c r="B38" s="118"/>
+      <c r="C38" s="118"/>
+      <c r="D38" s="118"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="93" t="s">
+        <v>325</v>
+      </c>
+      <c r="C40" s="93" t="s">
+        <v>101</v>
+      </c>
+      <c r="D40" s="93" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="94" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="94" t="s">
+        <v>453</v>
+      </c>
+      <c r="C41" s="94" t="s">
+        <v>454</v>
+      </c>
+      <c r="D41" s="94" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="94" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" s="94" t="s">
+        <v>456</v>
+      </c>
+      <c r="C42" s="94" t="s">
+        <v>457</v>
+      </c>
+      <c r="D42" s="94" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="94" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="94" t="s">
+        <v>459</v>
+      </c>
+      <c r="C43" s="94" t="s">
+        <v>460</v>
+      </c>
+      <c r="D43" s="94" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="94" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="94" t="s">
+        <v>462</v>
+      </c>
+      <c r="C44" s="94" t="s">
+        <v>463</v>
+      </c>
+      <c r="D44" s="94" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="118" t="s">
+        <v>465</v>
+      </c>
+      <c r="B47" s="118"/>
+      <c r="C47" s="118"/>
+      <c r="D47" s="118"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B49" s="93" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" s="93" t="s">
+        <v>113</v>
+      </c>
+      <c r="D49" s="93" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="116" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" s="116">
+        <v>8.2439999999999998</v>
+      </c>
+      <c r="C50" s="116">
+        <v>6.2960000000000003</v>
+      </c>
+      <c r="D50" s="159">
+        <v>14.54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="116" t="s">
+        <v>47</v>
+      </c>
+      <c r="B51" s="116">
+        <v>44.603999999999999</v>
+      </c>
+      <c r="C51" s="116">
+        <v>34.076000000000001</v>
+      </c>
+      <c r="D51" s="159">
+        <v>78.680000000000007</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="116" t="s">
+        <v>53</v>
+      </c>
+      <c r="B52" s="116">
+        <v>153.696</v>
+      </c>
+      <c r="C52" s="116">
+        <v>117.408</v>
+      </c>
+      <c r="D52" s="159">
+        <v>271.10399999999998</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="116" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53" s="116">
+        <v>735.75599999999997</v>
+      </c>
+      <c r="C53" s="116">
+        <v>561.85199999999998</v>
+      </c>
+      <c r="D53" s="159" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="118" t="s">
+        <v>467</v>
+      </c>
+      <c r="B56" s="118"/>
+      <c r="C56" s="118"/>
+      <c r="D56" s="118"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" s="93" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58" s="93" t="s">
+        <v>358</v>
+      </c>
+      <c r="C58" s="93" t="s">
+        <v>149</v>
+      </c>
+      <c r="D58" s="93" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" s="116" t="s">
+        <v>359</v>
+      </c>
+      <c r="B59" s="116" t="s">
+        <v>468</v>
+      </c>
+      <c r="C59" s="116" t="s">
+        <v>469</v>
+      </c>
+      <c r="D59" s="116" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="116" t="s">
+        <v>363</v>
+      </c>
+      <c r="B60" s="116">
+        <v>17</v>
+      </c>
+      <c r="C60" s="116">
+        <v>14</v>
+      </c>
+      <c r="D60" s="116"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="116" t="s">
+        <v>364</v>
+      </c>
+      <c r="B61" s="116" t="s">
+        <v>471</v>
+      </c>
+      <c r="C61" s="116" t="s">
+        <v>472</v>
+      </c>
+      <c r="D61" s="116" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="36" x14ac:dyDescent="0.35">
+      <c r="A62" s="116" t="s">
+        <v>209</v>
+      </c>
+      <c r="B62" s="116" t="s">
+        <v>474</v>
+      </c>
+      <c r="C62" s="116" t="s">
+        <v>474</v>
+      </c>
+      <c r="D62" s="116" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="36" x14ac:dyDescent="0.35">
+      <c r="A63" s="116" t="s">
+        <v>476</v>
+      </c>
+      <c r="B63" s="159" t="s">
+        <v>477</v>
+      </c>
+      <c r="C63" s="159" t="s">
+        <v>477</v>
+      </c>
+      <c r="D63" s="116"/>
+    </row>
+    <row r="64" spans="1:4" ht="36" x14ac:dyDescent="0.35">
+      <c r="A64" s="159" t="s">
+        <v>478</v>
+      </c>
+      <c r="B64" s="159" t="s">
+        <v>479</v>
+      </c>
+      <c r="C64" s="159" t="s">
+        <v>480</v>
+      </c>
+      <c r="D64" s="116" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="118" t="s">
+        <v>507</v>
+      </c>
+      <c r="B67" s="118"/>
+      <c r="C67" s="118"/>
+      <c r="D67" s="118"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" s="93" t="s">
+        <v>9</v>
+      </c>
+      <c r="B69" s="93" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="93" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="36" x14ac:dyDescent="0.35">
+      <c r="A70" s="94" t="s">
+        <v>369</v>
+      </c>
+      <c r="B70" s="94" t="s">
+        <v>482</v>
+      </c>
+      <c r="C70" s="94" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" s="94" t="s">
+        <v>269</v>
+      </c>
+      <c r="B71" s="94" t="s">
+        <v>372</v>
+      </c>
+      <c r="C71" s="94"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" s="94" t="s">
+        <v>483</v>
+      </c>
+      <c r="B72" s="94" t="s">
+        <v>376</v>
+      </c>
+      <c r="C72" s="94"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" s="94" t="s">
+        <v>484</v>
+      </c>
+      <c r="B73" s="94" t="s">
+        <v>379</v>
+      </c>
+      <c r="C73" s="94"/>
+    </row>
+    <row r="74" spans="1:7" ht="36" x14ac:dyDescent="0.35">
+      <c r="A74" s="94" t="s">
+        <v>485</v>
+      </c>
+      <c r="B74" s="94" t="s">
+        <v>486</v>
+      </c>
+      <c r="C74" s="94"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" s="118" t="s">
+        <v>508</v>
+      </c>
+      <c r="B78" s="118"/>
+      <c r="C78" s="118"/>
+      <c r="D78" s="118"/>
+      <c r="E78" s="118"/>
+      <c r="F78" s="118"/>
+      <c r="G78" s="118"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B80" s="93" t="s">
+        <v>337</v>
+      </c>
+      <c r="C80" s="93" t="s">
+        <v>338</v>
+      </c>
+      <c r="D80" s="93" t="s">
+        <v>339</v>
+      </c>
+      <c r="E80" s="93" t="s">
+        <v>487</v>
+      </c>
+      <c r="F80" s="93" t="s">
+        <v>488</v>
+      </c>
+      <c r="G80" s="93" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="36" x14ac:dyDescent="0.35">
+      <c r="A81" s="157" t="s">
+        <v>41</v>
+      </c>
+      <c r="B81" s="157">
+        <v>12.41</v>
+      </c>
+      <c r="C81" s="157" t="s">
+        <v>489</v>
+      </c>
+      <c r="D81" s="157">
+        <v>6.2050000000000001</v>
+      </c>
+      <c r="E81" s="157">
+        <v>1.08</v>
+      </c>
+      <c r="F81" s="158" t="s">
+        <v>490</v>
+      </c>
+      <c r="G81" s="158" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" s="157" t="s">
+        <v>47</v>
+      </c>
+      <c r="B82" s="157">
+        <v>67.16</v>
+      </c>
+      <c r="C82" s="157">
+        <v>3.3580000000000001</v>
+      </c>
+      <c r="D82" s="157">
+        <v>33.58</v>
+      </c>
+      <c r="E82" s="157">
+        <v>1.08</v>
+      </c>
+      <c r="F82" s="158">
+        <v>4.4379999999999997</v>
+      </c>
+      <c r="G82" s="158" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" s="157" t="s">
+        <v>53</v>
+      </c>
+      <c r="B83" s="157">
+        <v>231.41</v>
+      </c>
+      <c r="C83" s="157" t="s">
+        <v>492</v>
+      </c>
+      <c r="D83" s="157">
+        <v>115.705</v>
+      </c>
+      <c r="E83" s="157">
+        <v>1.08</v>
+      </c>
+      <c r="F83" s="158" t="s">
+        <v>493</v>
+      </c>
+      <c r="G83" s="158" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" s="157" t="s">
+        <v>58</v>
+      </c>
+      <c r="B84" s="157" t="s">
+        <v>495</v>
+      </c>
+      <c r="C84" s="157" t="s">
+        <v>496</v>
+      </c>
+      <c r="D84" s="157">
+        <v>553.70500000000004</v>
+      </c>
+      <c r="E84" s="157">
+        <v>1.08</v>
+      </c>
+      <c r="F84" s="158" t="s">
+        <v>497</v>
+      </c>
+      <c r="G84" s="158" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" s="119" t="s">
+        <v>510</v>
+      </c>
+      <c r="B87" s="119"/>
+      <c r="C87" s="119"/>
+      <c r="D87" s="119"/>
+      <c r="E87" s="119"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A89" s="93" t="s">
+        <v>33</v>
+      </c>
+      <c r="B89" s="93" t="s">
+        <v>499</v>
+      </c>
+      <c r="C89" s="93" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" s="157" t="s">
+        <v>47</v>
+      </c>
+      <c r="B90" s="157" t="s">
+        <v>501</v>
+      </c>
+      <c r="C90" s="157" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A91" s="157" t="s">
+        <v>53</v>
+      </c>
+      <c r="B91" s="157">
+        <v>66</v>
+      </c>
+      <c r="C91" s="157" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A92" s="157" t="s">
+        <v>58</v>
+      </c>
+      <c r="B92" s="157">
+        <v>330</v>
+      </c>
+      <c r="C92" s="157" t="s">
+        <v>504</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A78:G78"/>
+    <mergeCell ref="A87:E87"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A47:D47"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="9">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>